<commit_message>
Note verified public data on GRB capacity and units; mark unverified RBI/FFS history
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HcbnVyHFWjMv5iL4iw2dZn
</commit_message>
<xml_diff>
--- a/RBI_Barrancabermeja/RBI_Barrancabermeja_ModeloEconomico.xlsx
+++ b/RBI_Barrancabermeja/RBI_Barrancabermeja_ModeloEconomico.xlsx
@@ -923,7 +923,7 @@
     <t xml:space="preserve">REFERENCIA DE PRODUCCIÓN – REFINERÍA: pérdida diaria si falla/para un equipo (SUPUESTOS ilustrativos salvo la capacidad, dato del usuario)</t>
   </si>
   <si>
-    <t xml:space="preserve">Capacidad refinería GRB (bpd) – dato del usuario</t>
+    <t xml:space="preserve">Capacidad refinería GRB (bpd): máx. 250.000 según prensa; 246.000 en 2024 [V]</t>
   </si>
   <si>
     <t xml:space="preserve">Precio del barril (USD/bbl) – SUPUESTO</t>
@@ -1972,11 +1972,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="99862709"/>
-        <c:axId val="93137468"/>
+        <c:axId val="98879776"/>
+        <c:axId val="77200317"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="99862709"/>
+        <c:axId val="98879776"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2042,7 +2042,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93137468"/>
+        <c:crossAx val="77200317"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2050,7 +2050,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="93137468"/>
+        <c:axId val="77200317"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2126,7 +2126,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="99862709"/>
+        <c:crossAx val="98879776"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2417,11 +2417,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="83704566"/>
-        <c:axId val="58409978"/>
+        <c:axId val="52859472"/>
+        <c:axId val="89450422"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="83704566"/>
+        <c:axId val="52859472"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2453,7 +2453,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58409978"/>
+        <c:crossAx val="89450422"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2461,7 +2461,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="58409978"/>
+        <c:axId val="89450422"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2503,7 +2503,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83704566"/>
+        <c:crossAx val="52859472"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>